<commit_message>
تعديل يدوي في شيت Card21 by admin at 2026-03-03 09:59:55
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -21506,7 +21506,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>1002</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -23796,16 +23796,56 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>3/3/2026</t>
@@ -23826,7 +23866,11 @@
           <t>م.رشدي،خبير نور الدين</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card5 by admin at 2026-03-07 21:17:24
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5294,71 +5294,19 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5391,56 +5339,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5458,71 +5370,19 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5540,11 +5400,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5560,51 +5416,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>1\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5627,66 +5451,26 @@
           <t>591</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>19\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5709,36 +5493,20 @@
           <t>758</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5749,26 +5517,10 @@
           <t>23\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5796,36 +5548,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>30/11/2025</t>
@@ -5836,21 +5564,9 @@
           <t>م.محمد عبدالله ،خبير.ارول</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5873,11 +5589,7 @@
           <t>895</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5888,51 +5600,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>13\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5955,41 +5635,21 @@
           <t>1055</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
@@ -6042,36 +5702,16 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>7/3/2026</t>
@@ -6092,11 +5732,7 @@
           <t>تم سن الفلاتس،تم تغير جريدتين خلفي240,320</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6114,71 +5750,19 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6196,71 +5780,19 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6268,56 +5800,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>11/2/2025</t>
@@ -6338,11 +5830,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6350,56 +5838,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -6420,11 +5868,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6432,56 +5876,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -6502,11 +5906,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6514,56 +5914,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>19/8/2025</t>
@@ -6584,11 +5944,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6596,56 +5952,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -6666,11 +5982,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6678,56 +5990,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>15\7\2024</t>
@@ -6738,21 +6010,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير جريد1</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6760,56 +6024,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>14\8\2024</t>
@@ -6820,21 +6044,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6842,56 +6058,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>30\9\2024</t>
@@ -6902,21 +6078,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تاكيد علي المعيار</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6924,56 +6092,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7006,56 +6134,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7066,21 +6154,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7088,56 +6168,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>30\1\2025</t>
@@ -7148,21 +6188,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7170,56 +6202,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>19\4\2025</t>
@@ -7230,21 +6222,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه ومعايره (1_2_4_5_7_8)</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7252,56 +6236,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -7322,11 +6266,7 @@
           <t>تم تغيير  زيت الجيربوكس</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7334,56 +6274,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>23\7\2025</t>
@@ -7404,11 +6304,7 @@
           <t>تم سن السليندر وتغيير الفلاتس وتغيير سير الفلاتس وتغيير جريد 1</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7416,56 +6312,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>13\10\2025</t>
@@ -7486,11 +6342,7 @@
           <t>تم تغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7498,56 +6350,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>30\11\2025</t>
@@ -7568,11 +6380,7 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7580,56 +6388,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -7650,11 +6418,7 @@
           <t>تم تغير سير  دوبل700(محمد نعيم)</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7662,56 +6426,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -7732,11 +6456,7 @@
           <t>تم تغير سوفت كرد لbc</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7744,56 +6464,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -7814,11 +6494,7 @@
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7826,56 +6502,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -7896,11 +6532,7 @@
           <t>تم تغيير  سير 1200 الدوفر المسنن للتجربه</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15718,7 +14350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15814,18 +14446,66 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15858,19 +14538,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>21\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15888,18 +14600,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15917,7 +14677,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -15933,22 +14697,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>27\1\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15971,25 +14759,61 @@
           <t>566</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>10\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16012,16 +14836,36 @@
           <t>737</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -16032,9 +14876,21 @@
           <t>16\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16062,12 +14918,36 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>23/11/2025</t>
@@ -16078,7 +14958,11 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -16106,7 +14990,11 @@
           <t>851</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -16117,18 +15005,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>22\9\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16151,21 +15067,41 @@
           <t>1059</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>22/1/2026</t>
@@ -16203,18 +15139,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16232,18 +15216,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16261,18 +15293,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16280,16 +15360,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>12/4/2025</t>
@@ -16317,16 +15437,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>31/5/2025</t>
@@ -16354,16 +15514,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -16391,16 +15591,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -16428,20 +15668,76 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16449,16 +15745,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>31/1/2026</t>
@@ -16486,16 +15822,56 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -16514,6 +15890,43 @@
       <c r="O20" t="inlineStr">
         <is>
           <t>يوسف وابراهيم</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>7/3/2026</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>قطع سير700</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>تم تغير سير 700(مشلان)</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>رضا</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card10 by admin at 2026-03-08 15:48:55
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -7859,18 +7859,66 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7888,7 +7936,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7899,19 +7951,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7929,18 +8013,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7958,7 +8090,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7974,22 +8110,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8012,25 +8172,61 @@
           <t>584</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8053,20 +8249,36 @@
           <t>753</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8077,9 +8289,21 @@
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8107,19 +8331,51 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.مصطفي</t>
@@ -8147,7 +8403,11 @@
           <t>887</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8158,18 +8418,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>8\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8187,18 +8475,66 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>8\3\2026</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>تم سن فلاتس وتغير جريدع علويه240 وجريده320</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8216,18 +8552,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8245,18 +8629,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8274,18 +8706,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8293,16 +8773,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -8330,16 +8850,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>4/5/2025</t>
@@ -8367,16 +8927,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>16/6/2025</t>
@@ -8404,16 +9004,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -8441,16 +9081,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -8478,16 +9158,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -8515,22 +9235,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجريده 1</t>
@@ -8548,22 +9312,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -8581,22 +9389,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
@@ -8614,22 +9466,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>تم تغييرالجرائد الاماميه (1_2_4_5_7_8) ومعايرها</t>
@@ -8647,16 +9543,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -8684,22 +9620,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>تم تغيير الفلاتس وتغيير جريده 1</t>
@@ -8717,16 +9697,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>8\10\2025</t>
@@ -8754,16 +9774,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>27\11\2025</t>
@@ -8791,16 +9851,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -8843,21 +9943,41 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>8/2/2026</t>
@@ -8885,16 +10005,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -14446,66 +15606,18 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14538,51 +15650,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>21\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14600,66 +15680,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14677,11 +15709,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -14697,46 +15725,22 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>27\1\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14759,61 +15763,25 @@
           <t>566</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>10\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14836,36 +15804,16 @@
           <t>737</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -14876,21 +15824,9 @@
           <t>16\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14918,36 +15854,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>23/11/2025</t>
@@ -14958,11 +15870,7 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -14990,11 +15898,7 @@
           <t>851</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -15005,46 +15909,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>22\9\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15067,41 +15943,21 @@
           <t>1059</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>22/1/2026</t>
@@ -15139,66 +15995,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15216,66 +16024,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -15293,66 +16053,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -15360,56 +16072,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>12/4/2025</t>
@@ -15437,56 +16109,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>31/5/2025</t>
@@ -15514,56 +16146,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -15591,56 +16183,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -15668,76 +16220,20 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15745,56 +16241,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>31/1/2026</t>
@@ -15822,56 +16278,16 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>18/2/2026</t>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card2 by admin at 2026-03-08 15:51:16
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -7859,66 +7859,18 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7936,11 +7888,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7951,51 +7899,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8013,66 +7929,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8090,11 +7958,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8110,46 +7974,22 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8172,61 +8012,25 @@
           <t>584</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8249,36 +8053,20 @@
           <t>753</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8289,21 +8077,9 @@
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8331,51 +8107,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.مصطفي</t>
@@ -8403,11 +8147,7 @@
           <t>887</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8418,46 +8158,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>8\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8475,46 +8187,22 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -8552,66 +8240,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8629,66 +8269,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8706,66 +8298,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8773,56 +8317,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -8850,56 +8354,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>4/5/2025</t>
@@ -8927,56 +8391,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>16/6/2025</t>
@@ -9004,56 +8428,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -9081,56 +8465,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -9158,56 +8502,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -9235,66 +8539,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجريده 1</t>
@@ -9312,66 +8572,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -9389,66 +8605,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
@@ -9466,66 +8638,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>تم تغييرالجرائد الاماميه (1_2_4_5_7_8) ومعايرها</t>
@@ -9543,56 +8671,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -9620,66 +8708,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>تم تغيير الفلاتس وتغيير جريده 1</t>
@@ -9697,56 +8741,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>8\10\2025</t>
@@ -9774,56 +8778,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>27\11\2025</t>
@@ -9851,56 +8815,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -9943,41 +8867,21 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>8/2/2026</t>
@@ -10005,56 +8909,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -19146,7 +18010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19242,21 +18106,61 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -19279,7 +18183,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19290,19 +18198,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -19320,7 +18260,11 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19336,18 +18280,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19365,18 +18337,66 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19399,25 +18419,61 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19440,16 +18496,36 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19460,9 +18536,21 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19485,7 +18573,11 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19496,17 +18588,41 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -19539,12 +18655,36 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -19555,7 +18695,11 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -19583,21 +18727,41 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -19635,18 +18799,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19664,18 +18876,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19693,18 +18953,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19712,16 +19020,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -19749,16 +19097,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -19786,16 +19174,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -19823,16 +19251,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -19860,16 +19328,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19897,16 +19405,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19934,16 +19482,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -19971,16 +19559,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -20010,16 +19638,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -20047,16 +19715,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -20075,6 +19783,43 @@
       <c r="O23" t="inlineStr">
         <is>
           <t>يوسف وابراهيم</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>8\3\2026</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>تجربه</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>تم تبديل اغطيه دوفر بكرد12</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>ابراهيم ,ناجي</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card12 by admin at 2026-03-08 15:51:28
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5193,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5294,19 +5294,71 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5339,20 +5391,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5370,19 +5458,71 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5400,7 +5540,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5416,19 +5560,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>1\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5451,26 +5627,66 @@
           <t>591</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>19\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5493,20 +5709,36 @@
           <t>758</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5517,10 +5749,26 @@
           <t>23\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5548,12 +5796,36 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>30/11/2025</t>
@@ -5564,9 +5836,21 @@
           <t>م.محمد عبدالله ،خبير.ارول</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5589,7 +5873,11 @@
           <t>895</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5600,19 +5888,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>13\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5635,21 +5955,41 @@
           <t>1055</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
@@ -5702,16 +6042,36 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>7/3/2026</t>
@@ -5732,7 +6092,11 @@
           <t>تم سن الفلاتس،تم تغير جريدتين خلفي240,320</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5750,19 +6114,71 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5780,19 +6196,71 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5800,16 +6268,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>11/2/2025</t>
@@ -5830,7 +6338,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5838,16 +6350,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -5868,7 +6420,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5876,16 +6432,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -5906,7 +6502,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5914,16 +6514,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>19/8/2025</t>
@@ -5944,7 +6584,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5952,16 +6596,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -5982,7 +6666,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5990,16 +6678,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>15\7\2024</t>
@@ -6010,13 +6738,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير جريد1</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6024,16 +6760,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>14\8\2024</t>
@@ -6044,13 +6820,21 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6058,16 +6842,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>30\9\2024</t>
@@ -6078,13 +6902,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تاكيد علي المعيار</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6092,16 +6924,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -6134,16 +7006,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -6154,13 +7066,21 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6168,16 +7088,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>30\1\2025</t>
@@ -6188,13 +7148,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6202,16 +7170,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>19\4\2025</t>
@@ -6222,13 +7230,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O25" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه ومعايره (1_2_4_5_7_8)</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6236,16 +7252,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -6266,7 +7322,11 @@
           <t>تم تغيير  زيت الجيربوكس</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6274,16 +7334,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>23\7\2025</t>
@@ -6304,7 +7404,11 @@
           <t>تم سن السليندر وتغيير الفلاتس وتغيير سير الفلاتس وتغيير جريد 1</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6312,16 +7416,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>13\10\2025</t>
@@ -6342,7 +7486,11 @@
           <t>تم تغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6350,16 +7498,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>30\11\2025</t>
@@ -6380,7 +7568,11 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6388,16 +7580,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -6418,7 +7650,11 @@
           <t>تم تغير سير  دوبل700(محمد نعيم)</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6426,16 +7662,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -6456,7 +7732,11 @@
           <t>تم تغير سوفت كرد لbc</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6464,16 +7744,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -6494,7 +7814,11 @@
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6502,16 +7826,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -6532,7 +7896,49 @@
           <t>تم تغيير  سير 1200 الدوفر المسنن للتجربه</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>8\3\2026</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>ابراهيم ,ناجي</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>تجربه</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>تم تبديل اغطيه دوفر بكرد12</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18106,61 +19512,21 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -18183,11 +19549,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18198,51 +19560,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18260,11 +19590,7 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18280,46 +19606,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18337,66 +19635,18 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18419,61 +19669,25 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18496,36 +19710,16 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18536,21 +19730,9 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18573,11 +19755,7 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18588,41 +19766,17 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -18655,36 +19809,12 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -18695,11 +19825,7 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -18727,41 +19853,21 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18799,66 +19905,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18876,66 +19934,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -18953,66 +19963,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19020,56 +19982,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -19097,56 +20019,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -19174,56 +20056,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -19251,56 +20093,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -19328,56 +20130,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19405,56 +20167,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19482,56 +20204,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -19559,56 +20241,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -19638,56 +20280,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -19715,56 +20317,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card10 by admin at 2026-03-09 15:43:16
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5294,71 +5294,19 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5391,56 +5339,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5458,71 +5370,19 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5540,11 +5400,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5560,51 +5416,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>1\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5627,66 +5451,26 @@
           <t>591</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>19\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5709,36 +5493,20 @@
           <t>758</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5749,26 +5517,10 @@
           <t>23\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5796,36 +5548,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>30/11/2025</t>
@@ -5836,21 +5564,9 @@
           <t>م.محمد عبدالله ،خبير.ارول</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5873,11 +5589,7 @@
           <t>895</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5888,51 +5600,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>13\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5955,41 +5635,21 @@
           <t>1055</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
@@ -6042,36 +5702,16 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>7/3/2026</t>
@@ -6092,11 +5732,7 @@
           <t>تم سن الفلاتس،تم تغير جريدتين خلفي240,320</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6114,71 +5750,19 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6196,71 +5780,19 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6268,56 +5800,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>11/2/2025</t>
@@ -6338,11 +5830,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6350,56 +5838,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -6420,11 +5868,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6432,56 +5876,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -6502,11 +5906,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6514,56 +5914,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>19/8/2025</t>
@@ -6584,11 +5944,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6596,56 +5952,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -6666,11 +5982,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6678,56 +5990,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>15\7\2024</t>
@@ -6738,21 +6010,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير جريد1</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6760,56 +6024,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>14\8\2024</t>
@@ -6820,21 +6044,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6842,56 +6058,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>30\9\2024</t>
@@ -6902,21 +6078,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تاكيد علي المعيار</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6924,56 +6092,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7006,56 +6134,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7066,21 +6154,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7088,56 +6168,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>30\1\2025</t>
@@ -7148,21 +6188,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7170,56 +6202,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>19\4\2025</t>
@@ -7230,21 +6222,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه ومعايره (1_2_4_5_7_8)</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7252,56 +6236,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -7322,11 +6266,7 @@
           <t>تم تغيير  زيت الجيربوكس</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7334,56 +6274,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>23\7\2025</t>
@@ -7404,11 +6304,7 @@
           <t>تم سن السليندر وتغيير الفلاتس وتغيير سير الفلاتس وتغيير جريد 1</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7416,56 +6312,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>13\10\2025</t>
@@ -7486,11 +6342,7 @@
           <t>تم تغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7498,56 +6350,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>30\11\2025</t>
@@ -7568,11 +6380,7 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7580,56 +6388,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -7650,11 +6418,7 @@
           <t>تم تغير سير  دوبل700(محمد نعيم)</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7662,56 +6426,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -7732,11 +6456,7 @@
           <t>تم تغير سوفت كرد لbc</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7744,56 +6464,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -7814,11 +6494,7 @@
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7826,56 +6502,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -7896,11 +6532,7 @@
           <t>تم تغيير  سير 1200 الدوفر المسنن للتجربه</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9265,18 +7897,66 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9294,7 +7974,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9305,19 +7989,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9335,18 +8051,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9364,7 +8128,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9380,22 +8148,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9418,25 +8210,61 @@
           <t>584</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9459,20 +8287,36 @@
           <t>753</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9483,9 +8327,21 @@
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9513,19 +8369,51 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.مصطفي</t>
@@ -9553,7 +8441,11 @@
           <t>887</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9564,18 +8456,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>8\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9593,22 +8513,46 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1150</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -9646,18 +8590,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9675,18 +8667,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9704,18 +8744,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9723,16 +8811,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -9760,16 +8888,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>4/5/2025</t>
@@ -9797,16 +8965,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>16/6/2025</t>
@@ -9834,16 +9042,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -9871,16 +9119,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -9908,16 +9196,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -9945,22 +9273,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجريده 1</t>
@@ -9978,22 +9350,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -10011,22 +9427,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
@@ -10044,22 +9504,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>تم تغييرالجرائد الاماميه (1_2_4_5_7_8) ومعايرها</t>
@@ -10077,16 +9581,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -10114,22 +9658,66 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>تم تغيير الفلاتس وتغيير جريده 1</t>
@@ -10147,16 +9735,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>8\10\2025</t>
@@ -10184,16 +9812,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>27\11\2025</t>
@@ -10221,16 +9889,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -10273,21 +9981,41 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>8/2/2026</t>
@@ -10315,16 +10043,56 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card10 by admin at 2026-03-09 18:42:13
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -7801,7 +7801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10111,6 +10111,43 @@
       <c r="O30" t="inlineStr">
         <is>
           <t>يوسف وابراهيم</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>8/3/2026</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>قطع سيى700</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>تم تغير سير700(مشلان)</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>رضا</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة صف جديد في Card2 by admin at 2026-03-10 09:29:14
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -7897,66 +7897,18 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7974,11 +7926,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7989,51 +7937,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8051,66 +7967,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8128,11 +7996,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8148,46 +8012,22 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8210,61 +8050,25 @@
           <t>584</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8287,36 +8091,20 @@
           <t>753</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8327,21 +8115,9 @@
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8369,51 +8145,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.مصطفي</t>
@@ -8441,11 +8185,7 @@
           <t>887</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -8456,46 +8196,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>8\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8523,36 +8235,16 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -8590,66 +8282,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8667,66 +8311,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8744,66 +8340,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8811,56 +8359,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -8888,56 +8396,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>4/5/2025</t>
@@ -8965,56 +8433,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>16/6/2025</t>
@@ -9042,56 +8470,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -9119,56 +8507,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -9196,56 +8544,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -9273,66 +8581,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>20\7\2024</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجريده 1</t>
@@ -9350,66 +8614,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -9427,66 +8647,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>6\3\2025</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
@@ -9504,66 +8680,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>14\4\2025</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>تم تغييرالجرائد الاماميه (1_2_4_5_7_8) ومعايرها</t>
@@ -9581,56 +8713,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -9658,66 +8750,22 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>20\7\2025</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>تم تغيير الفلاتس وتغيير جريده 1</t>
@@ -9735,56 +8783,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>8\10\2025</t>
@@ -9812,56 +8820,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>27\11\2025</t>
@@ -9889,56 +8857,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -9981,41 +8909,21 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>8/2/2026</t>
@@ -10043,56 +8951,16 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -19221,7 +18089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19317,21 +18185,61 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -19354,7 +18262,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19365,19 +18277,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -19395,7 +18339,11 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19411,18 +18359,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19440,18 +18416,66 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19474,25 +18498,61 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19515,16 +18575,36 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19535,9 +18615,21 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19560,7 +18652,11 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -19571,17 +18667,41 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -19614,12 +18734,36 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -19630,7 +18774,11 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -19658,21 +18806,41 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -19710,18 +18878,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19739,18 +18955,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19768,18 +19032,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19787,16 +19099,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -19824,16 +19176,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -19861,16 +19253,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -19898,16 +19330,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -19935,16 +19407,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19972,16 +19484,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -20009,16 +19561,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -20046,16 +19638,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -20085,16 +19717,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -20122,16 +19794,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -20159,16 +19871,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -20187,6 +19939,67 @@
       <c r="O24" t="inlineStr">
         <is>
           <t>ابراهيم ,ناجي</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1150</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1141</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>10/3/2026</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سيرفيس </t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم سن دوفر 2شوط وتغير جريده خلفيه 240و320وسن فلاتس </t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>م.عبدالله،حسام ،محمود ايهاب</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card18 by admin at 2026-03-11 09:25:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -18185,61 +18185,21 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -18262,11 +18222,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18277,51 +18233,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18339,11 +18263,7 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18359,46 +18279,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18416,66 +18308,18 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18498,61 +18342,25 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18575,36 +18383,16 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18615,21 +18403,9 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18652,11 +18428,7 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18667,41 +18439,17 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -18734,36 +18482,12 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -18774,11 +18498,7 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -18806,41 +18526,21 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18878,66 +18578,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18955,66 +18607,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19032,66 +18636,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19099,56 +18655,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -19176,56 +18692,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -19253,56 +18729,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -19330,56 +18766,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -19407,56 +18803,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19484,56 +18840,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19561,56 +18877,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -19638,56 +18914,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -19717,56 +18953,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -19794,56 +18990,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -19871,56 +19027,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -25928,7 +25044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26034,20 +25150,76 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -26065,28 +25237,76 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>1\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -26104,20 +25324,76 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -26135,8 +25411,16 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -26147,20 +25431,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>11\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -26183,9 +25503,21 @@
           <t>590</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -26196,18 +25528,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>29\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -26230,27 +25590,71 @@
           <t>785</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>20\8\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -26273,7 +25677,11 @@
           <t>883</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -26284,20 +25692,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>23\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -26315,20 +25759,76 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -26346,20 +25846,76 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -26377,20 +25933,76 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -26408,20 +26020,76 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -26429,23 +26097,71 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل</t>
@@ -26456,7 +26172,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -26464,23 +26184,71 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr">
         <is>
           <t>تم سير مضرب dfk 25*1.5*974 flat</t>
@@ -26491,7 +26259,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -26499,23 +26271,71 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>1\12\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
           <t>تم سن الفلاتس +صيانه نصف سنويه</t>
@@ -26526,7 +26346,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -26534,23 +26358,71 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>10\3\2025</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -26561,7 +26433,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -26569,16 +26445,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>29\4\2025</t>
@@ -26589,7 +26505,11 @@
           <t>590.1</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O17" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه (1_2_4__5_7_8) ومعيارته وسن السليندر</t>
@@ -26600,7 +26520,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -26608,16 +26532,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>14\8\2025</t>
@@ -26628,7 +26592,11 @@
           <t>9736 h   775 t</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>تم تغيير زيت الجيربوكس</t>
@@ -26639,7 +26607,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -26647,16 +26619,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>20\8\2025</t>
@@ -26667,7 +26679,11 @@
           <t>785 t</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم تغيير جريده1  وجريده اليكران(90)</t>
@@ -26678,7 +26694,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -26686,16 +26706,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>23\10\2025</t>
@@ -26706,7 +26766,11 @@
           <t>883 t</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تغيير الجرئد الخلفيه (1_5_8) ومعارته</t>
@@ -26717,7 +26781,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -26725,16 +26793,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/4/2025</t>
@@ -26745,7 +26853,11 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تغير سير 1270</t>
@@ -26756,7 +26868,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -26764,16 +26880,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>29/6/2025</t>
@@ -26784,7 +26940,11 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O22" t="inlineStr">
         <is>
           <t>تم تغير سير 1270</t>
@@ -26795,7 +26955,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -26803,16 +26967,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -26823,7 +27027,11 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم تغير سير 1270(ميجا فلكس)</t>
@@ -26834,7 +27042,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -26842,16 +27054,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -26862,7 +27114,11 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم تغير سير 1270(محمد نعيم)</t>
@@ -26873,7 +27129,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -26881,16 +27141,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>28\10\2025</t>
@@ -26901,7 +27201,11 @@
           <t>تم تركيب مساحه خروج شريط(35*26*1)</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O25" t="inlineStr">
         <is>
           <t>كسر مساحه خروج شريط</t>
@@ -26912,7 +27216,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -26935,20 +27243,36 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -26964,7 +27288,11 @@
           <t xml:space="preserve">سيرفيس </t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O26" t="inlineStr">
         <is>
           <t>تم تغير فلاتس متحركه وتم تغير اول جريده 240وتم تغير 12جريده 550ع عيار 14ساو</t>
@@ -26987,16 +27315,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>12/1/2026</t>
@@ -27007,7 +27375,11 @@
           <t>صوت وفايبريشن عالي  ف مجموعه دليفري وبعد  معاينه وجد تاكل ف طاره عصاره خروج شريط</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>تم تركيب الطاره عكس اتجاها لحين تصنيع طاره أخري وتم تنظيف رولين سير700</t>
@@ -27018,30 +27390,98 @@
           <t>م.محمد عبدالله ،محمود ايهاب،،سلامه،ابراهيم،مصطفي</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،محمود ايهاب،،سلامه،ابراهيم،مصطفي</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -27049,16 +27489,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>15/1/2026</t>
@@ -27069,7 +27549,11 @@
           <t>قطع سير700</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O29" t="inlineStr">
         <is>
           <t>تم تغير سير700(مشلان)</t>
@@ -27080,7 +27564,11 @@
           <t>مصطفي</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -27088,16 +27576,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>30/1/2026</t>
@@ -27108,7 +27636,11 @@
           <t>انقطاع سير1800</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr">
         <is>
           <t>تم تغير سير1800</t>
@@ -27119,7 +27651,11 @@
           <t>سلامه</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -27127,16 +27663,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>31/1/2026</t>
@@ -27147,7 +27723,11 @@
           <t>انقطاع سير دوفر 1200</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
           <t>تم تغير سير دوفر 1200</t>
@@ -27158,7 +27738,11 @@
           <t>عمر</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -27166,16 +27750,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>1/2/2026</t>
@@ -27186,7 +27810,11 @@
           <t>انقطاع سير دوفر 1200</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O32" t="inlineStr">
         <is>
           <t>تم تغير سير دوفر 1200</t>
@@ -27197,7 +27825,11 @@
           <t>عمر</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -27205,16 +27837,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -27225,7 +27897,11 @@
           <t>تشحيم</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
@@ -27236,7 +27912,11 @@
           <t>مصطفى</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -27244,16 +27924,56 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>28/2/2026</t>
@@ -27264,7 +27984,11 @@
           <t>قطع سير الكويلر1465</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr">
         <is>
           <t>تم تغير سير فلات 1465</t>
@@ -27275,7 +27999,50 @@
           <t>رضا</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>11/3/2026</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>هلك سير1270</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>تم تغير سير1270(مشلان)</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card2 by admin at 2026-03-11 09:27:04
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -18089,7 +18089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18185,21 +18185,61 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -18222,7 +18262,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18233,19 +18277,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18263,7 +18339,11 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18279,18 +18359,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18308,18 +18416,66 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18342,25 +18498,61 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18383,16 +18575,36 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18403,9 +18615,21 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18428,7 +18652,11 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18439,17 +18667,41 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -18482,12 +18734,36 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -18498,7 +18774,11 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -18526,21 +18806,41 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18578,18 +18878,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18607,18 +18955,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -18636,18 +19032,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -18655,16 +19099,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -18692,16 +19176,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -18729,16 +19253,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -18766,16 +19330,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -18803,16 +19407,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -18840,16 +19484,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -18877,16 +19561,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -18914,16 +19638,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18953,16 +19717,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -18990,16 +19794,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -19027,16 +19871,56 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -19084,20 +19968,36 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>10/3/2026</t>
@@ -19116,6 +20016,43 @@
       <c r="O25" t="inlineStr">
         <is>
           <t>م.عبدالله،حسام ،محمود ايهاب</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>9/3/2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>كسر جلبه بليه</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>تم تغير جلبه بليه</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>مصطفى ،عمر</t>
         </is>
       </c>
     </row>
@@ -25150,76 +26087,20 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -25237,76 +26118,28 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>1\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -25324,76 +26157,20 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -25411,16 +26188,8 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -25431,56 +26200,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>11\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -25503,21 +26236,9 @@
           <t>590</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -25528,46 +26249,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>29\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -25590,71 +26283,27 @@
           <t>785</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>20\8\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25677,11 +26326,7 @@
           <t>883</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -25692,56 +26337,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>23\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -25759,76 +26368,20 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -25846,76 +26399,20 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25933,76 +26430,20 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -26020,76 +26461,20 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -26097,71 +26482,23 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل</t>
@@ -26172,11 +26509,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -26184,71 +26517,23 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
           <t>تم سير مضرب dfk 25*1.5*974 flat</t>
@@ -26259,11 +26544,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -26271,71 +26552,23 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>1\12\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>تم سن الفلاتس +صيانه نصف سنويه</t>
@@ -26346,11 +26579,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -26358,71 +26587,23 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>10\3\2025</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -26433,11 +26614,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -26445,56 +26622,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>29\4\2025</t>
@@ -26505,11 +26642,7 @@
           <t>590.1</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه (1_2_4__5_7_8) ومعيارته وسن السليندر</t>
@@ -26520,11 +26653,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -26532,56 +26661,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>14\8\2025</t>
@@ -26592,11 +26681,7 @@
           <t>9736 h   775 t</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
           <t>تم تغيير زيت الجيربوكس</t>
@@ -26607,11 +26692,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -26619,56 +26700,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>20\8\2025</t>
@@ -26679,11 +26720,7 @@
           <t>785 t</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم تغيير جريده1  وجريده اليكران(90)</t>
@@ -26694,11 +26731,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -26706,56 +26739,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>23\10\2025</t>
@@ -26766,11 +26759,7 @@
           <t>883 t</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تغيير الجرئد الخلفيه (1_5_8) ومعارته</t>
@@ -26781,11 +26770,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -26793,56 +26778,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/4/2025</t>
@@ -26853,11 +26798,7 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تغير سير 1270</t>
@@ -26868,11 +26809,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -26880,56 +26817,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>29/6/2025</t>
@@ -26940,11 +26837,7 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
           <t>تم تغير سير 1270</t>
@@ -26955,11 +26848,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -26967,56 +26856,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>30/9/2025</t>
@@ -27027,11 +26876,7 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم تغير سير 1270(ميجا فلكس)</t>
@@ -27042,11 +26887,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -27054,56 +26895,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -27114,11 +26915,7 @@
           <t>قطع سير كويلر مسنن 1270</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم تغير سير 1270(محمد نعيم)</t>
@@ -27129,11 +26926,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -27141,56 +26934,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>28\10\2025</t>
@@ -27201,11 +26954,7 @@
           <t>تم تركيب مساحه خروج شريط(35*26*1)</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>كسر مساحه خروج شريط</t>
@@ -27216,11 +26965,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -27243,36 +26988,20 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -27288,11 +27017,7 @@
           <t xml:space="preserve">سيرفيس </t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>تم تغير فلاتس متحركه وتم تغير اول جريده 240وتم تغير 12جريده 550ع عيار 14ساو</t>
@@ -27315,56 +27040,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>12/1/2026</t>
@@ -27375,11 +27060,7 @@
           <t>صوت وفايبريشن عالي  ف مجموعه دليفري وبعد  معاينه وجد تاكل ف طاره عصاره خروج شريط</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>تم تركيب الطاره عكس اتجاها لحين تصنيع طاره أخري وتم تنظيف رولين سير700</t>
@@ -27390,98 +27071,30 @@
           <t>م.محمد عبدالله ،محمود ايهاب،،سلامه،ابراهيم،مصطفي</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،محمود ايهاب،،سلامه،ابراهيم،مصطفي</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -27489,56 +27102,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>15/1/2026</t>
@@ -27549,11 +27122,7 @@
           <t>قطع سير700</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
           <t>تم تغير سير700(مشلان)</t>
@@ -27564,11 +27133,7 @@
           <t>مصطفي</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -27576,56 +27141,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>30/1/2026</t>
@@ -27636,11 +27161,7 @@
           <t>انقطاع سير1800</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
           <t>تم تغير سير1800</t>
@@ -27651,11 +27172,7 @@
           <t>سلامه</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -27663,56 +27180,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>31/1/2026</t>
@@ -27723,11 +27200,7 @@
           <t>انقطاع سير دوفر 1200</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
           <t>تم تغير سير دوفر 1200</t>
@@ -27738,11 +27211,7 @@
           <t>عمر</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -27750,56 +27219,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>1/2/2026</t>
@@ -27810,11 +27239,7 @@
           <t>انقطاع سير دوفر 1200</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
           <t>تم تغير سير دوفر 1200</t>
@@ -27825,11 +27250,7 @@
           <t>عمر</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -27837,56 +27258,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -27897,11 +27278,7 @@
           <t>تشحيم</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
@@ -27912,11 +27289,7 @@
           <t>مصطفى</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -27924,56 +27297,16 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>28/2/2026</t>
@@ -27984,11 +27317,7 @@
           <t>قطع سير الكويلر1465</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
           <t>تم تغير سير فلات 1465</t>
@@ -27999,11 +27328,7 @@
           <t>رضا</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">

</xml_diff>

<commit_message>
إضافة حدث جديد في Card1 by admin at 2026-03-14 06:17:12
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -17120,7 +17120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17216,14 +17216,46 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>1/2/2024</t>
@@ -17234,7 +17266,11 @@
           <t>تم تشغيل الماكينه اول مره</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>زكريا</t>
@@ -17272,19 +17308,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17302,14 +17370,46 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>11\8\2024</t>
@@ -17347,14 +17447,46 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>29\9\2024</t>
@@ -17392,20 +17524,56 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>22\12\2024</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>صيانه نصف سنويه</t>
@@ -17433,18 +17601,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17462,7 +17678,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17478,22 +17698,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>29\1\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17516,29 +17760,61 @@
           <t>565</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>5\4\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17561,16 +17837,36 @@
           <t>724</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17581,9 +17877,21 @@
           <t>5\7\2025</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17606,25 +17914,61 @@
           <t>859</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>24\9\2025</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17647,17 +17991,41 @@
           <t>1020</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>30/12/2025</t>
@@ -17695,18 +18063,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17724,18 +18140,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17753,18 +18217,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -17772,16 +18284,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -17809,16 +18361,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>30/8/2025</t>
@@ -17846,16 +18438,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -17898,17 +18530,41 @@
           <t>1094</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>4/2/2026</t>
@@ -17936,16 +18592,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>9/2/2026</t>
@@ -17973,16 +18669,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -18010,16 +18746,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>23/2/2026</t>
@@ -18047,16 +18823,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -18075,6 +18891,43 @@
       <c r="O23" t="inlineStr">
         <is>
           <t>رضا</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>28/10/2025</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>تم سن فلاتس وتغير جريده رقم 240</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>م.صيام،م.عبدالله</t>
         </is>
       </c>
     </row>
@@ -18185,61 +19038,21 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>تم الشتغيل</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>A.Elshenawy</t>
@@ -18262,11 +19075,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18277,51 +19086,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18339,11 +19116,7 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18359,46 +19132,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>27\2\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18416,66 +19161,18 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18498,61 +19195,25 @@
           <t>559</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>7\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18575,36 +19236,16 @@
           <t>727</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18615,21 +19256,9 @@
           <t>6\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18652,11 +19281,7 @@
           <t>860</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -18667,41 +19292,17 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>28\9\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله</t>
@@ -18734,36 +19335,12 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>1\11\2025</t>
@@ -18774,11 +19351,7 @@
           <t xml:space="preserve">تم سن فلاتس وعياره </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
@@ -18806,41 +19379,21 @@
           <t>1060</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18878,66 +19431,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18955,66 +19460,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19032,66 +19489,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19099,56 +19508,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -19176,56 +19545,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>22/10/2025</t>
@@ -19253,56 +19582,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -19330,56 +19619,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>15/11/2025</t>
@@ -19407,56 +19656,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19484,56 +19693,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>11/12/2025</t>
@@ -19561,56 +19730,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/1/2026</t>
@@ -19638,56 +19767,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -19717,56 +19806,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -19794,56 +19843,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -19871,56 +19880,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -19968,36 +19937,20 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>10/3/2026</t>

</xml_diff>

<commit_message>
إضافة صف جديد في Card1 by admin at 2026-03-14 06:19:47
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -17120,7 +17120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18900,16 +18900,56 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -18926,6 +18966,63 @@
         </is>
       </c>
       <c r="O24" t="inlineStr">
+        <is>
+          <t>م.صيام،م.عبدالله</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>851</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>918</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سيرفيس </t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>تم سن فلاتس وتغير اول جريده خلفيه 240</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>م.صيام،م.عبدالله</t>
         </is>

</xml_diff>

<commit_message>
تعديل حدث في Card1 - الصف 22 by admin at 2026-03-14 06:21:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -19002,11 +19002,31 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>28/10/2026</t>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card1 by admin at 2026-03-14 15:35:18
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -18065,62 +18065,62 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>1160</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>14/3/2026</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>سيرفيس</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>تم تغير جريده خلفيه 240و320</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t xml:space="preserve">حسام،م.محمد عبدالله </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card12 by admin at 2026-03-16 09:52:59
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5193,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5294,19 +5294,71 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5339,20 +5391,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5370,19 +5458,71 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5400,7 +5540,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5416,19 +5560,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>1\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5451,26 +5627,66 @@
           <t>591</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>19\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5493,20 +5709,36 @@
           <t>758</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5517,10 +5749,26 @@
           <t>23\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5548,12 +5796,36 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>30/11/2025</t>
@@ -5564,9 +5836,21 @@
           <t>م.محمد عبدالله ،خبير.ارول</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5589,7 +5873,11 @@
           <t>895</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5600,19 +5888,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>13\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5635,21 +5955,41 @@
           <t>1055</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
@@ -5702,16 +6042,36 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>7/3/2026</t>
@@ -5732,7 +6092,11 @@
           <t>تم سن الفلاتس،تم تغير جريدتين خلفي240,320</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5750,19 +6114,71 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5780,19 +6196,71 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5800,16 +6268,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>11/2/2025</t>
@@ -5830,7 +6338,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5838,16 +6350,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -5868,7 +6420,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5876,16 +6432,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -5906,7 +6502,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5914,16 +6514,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>19/8/2025</t>
@@ -5944,7 +6584,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5952,16 +6596,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -5982,7 +6666,11 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5990,16 +6678,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>15\7\2024</t>
@@ -6010,13 +6738,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير جريد1</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6024,16 +6760,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>14\8\2024</t>
@@ -6044,13 +6820,21 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6058,16 +6842,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>30\9\2024</t>
@@ -6078,13 +6902,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تاكيد علي المعيار</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6092,16 +6924,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -6134,16 +7006,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -6154,13 +7066,21 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6168,16 +7088,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>30\1\2025</t>
@@ -6188,13 +7148,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6202,16 +7170,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>19\4\2025</t>
@@ -6222,13 +7230,21 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O25" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه ومعايره (1_2_4_5_7_8)</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6236,16 +7252,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -6266,7 +7322,11 @@
           <t>تم تغيير  زيت الجيربوكس</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6274,16 +7334,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>23\7\2025</t>
@@ -6304,7 +7404,11 @@
           <t>تم سن السليندر وتغيير الفلاتس وتغيير سير الفلاتس وتغيير جريد 1</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6312,16 +7416,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>13\10\2025</t>
@@ -6342,7 +7486,11 @@
           <t>تم تغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6350,16 +7498,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>30\11\2025</t>
@@ -6380,7 +7568,11 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6388,16 +7580,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -6418,7 +7650,11 @@
           <t>تم تغير سير  دوبل700(محمد نعيم)</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6426,16 +7662,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -6456,7 +7732,11 @@
           <t>تم تغير سوفت كرد لbc</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6464,16 +7744,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -6494,7 +7814,11 @@
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6502,16 +7826,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -6532,7 +7896,11 @@
           <t>تم تغيير  سير 1200 الدوفر المسنن للتجربه</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6540,16 +7908,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -6570,7 +7978,49 @@
           <t>تم تبديل اغطيه دوفر بكرد12</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>16/3/2026</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>عمر</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>قطع سير1200</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>تم تغير سير1200</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17216,46 +18666,14 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>1/2/2024</t>
@@ -17266,11 +18684,7 @@
           <t>تم تشغيل الماكينه اول مره</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>زكريا</t>
@@ -17308,51 +18722,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17370,46 +18752,14 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>11\8\2024</t>
@@ -17447,46 +18797,14 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>29\9\2024</t>
@@ -17524,56 +18842,20 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>22\12\2024</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>صيانه نصف سنويه</t>
@@ -17601,66 +18883,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17678,11 +18912,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17698,46 +18928,22 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>29\1\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17760,61 +18966,29 @@
           <t>565</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>5\4\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17837,36 +19011,16 @@
           <t>724</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17877,21 +19031,9 @@
           <t>5\7\2025</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17914,61 +19056,25 @@
           <t>859</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>24\9\2025</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17991,41 +19097,17 @@
           <t>1020</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>30/12/2025</t>
@@ -18068,41 +19150,17 @@
           <t>1160</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>14/3/2026</t>
@@ -18140,66 +19198,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -18217,66 +19227,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -18284,56 +19246,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>30/6/2025</t>
@@ -18361,56 +19283,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>30/8/2025</t>
@@ -18438,56 +19320,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -18530,41 +19372,17 @@
           <t>1094</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>4/2/2026</t>
@@ -18592,56 +19410,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>9/2/2026</t>
@@ -18669,56 +19447,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -18746,56 +19484,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>23/2/2026</t>
@@ -18823,56 +19521,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -18900,56 +19558,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>28/10/2025</t>
@@ -19002,31 +19620,11 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>28/10/2026</t>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card12 by admin at 2026-03-16 09:53:18
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5193,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7990,16 +7990,56 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>16/3/2026</t>
@@ -8020,7 +8060,49 @@
           <t>تم تغير سير1200</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>16/3/2026</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>عمر</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>قطع سير700</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>تم تغير سير700</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card3 by admin at 2026-03-16 09:54:50
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -5294,71 +5294,19 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5391,56 +5339,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>15\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5458,71 +5370,19 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5540,11 +5400,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5560,51 +5416,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>1\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5627,66 +5451,26 @@
           <t>591</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>19\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5709,36 +5493,20 @@
           <t>758</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5749,26 +5517,10 @@
           <t>23\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5796,36 +5548,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>30/11/2025</t>
@@ -5836,21 +5564,9 @@
           <t>م.محمد عبدالله ،خبير.ارول</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5873,11 +5589,7 @@
           <t>895</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -5888,51 +5600,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>13\10\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5955,41 +5635,21 @@
           <t>1055</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
@@ -6042,36 +5702,16 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>7/3/2026</t>
@@ -6092,11 +5732,7 @@
           <t>تم سن الفلاتس،تم تغير جريدتين خلفي240,320</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6114,71 +5750,19 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6196,71 +5780,19 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6268,56 +5800,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>11/2/2025</t>
@@ -6338,11 +5830,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6350,56 +5838,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -6420,11 +5868,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6432,56 +5876,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -6502,11 +5906,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6514,56 +5914,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>19/8/2025</t>
@@ -6584,11 +5944,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6596,56 +5952,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -6666,11 +5982,7 @@
           <t>تم تغير سير 1270</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6678,56 +5990,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>15\7\2024</t>
@@ -6738,21 +6010,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير جريد1</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6760,56 +6024,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>14\8\2024</t>
@@ -6820,21 +6044,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6842,56 +6058,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>30\9\2024</t>
@@ -6902,21 +6078,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>تم تاكيد علي المعيار</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6924,56 +6092,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7006,56 +6134,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>15\10\2024</t>
@@ -7066,21 +6154,13 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7088,56 +6168,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>30\1\2025</t>
@@ -7148,21 +6188,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7170,56 +6202,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>19\4\2025</t>
@@ -7230,21 +6222,13 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه ومعايره (1_2_4_5_7_8)</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7252,56 +6236,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>10\7\2025</t>
@@ -7322,11 +6266,7 @@
           <t>تم تغيير  زيت الجيربوكس</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7334,56 +6274,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>23\7\2025</t>
@@ -7404,11 +6304,7 @@
           <t>تم سن السليندر وتغيير الفلاتس وتغيير سير الفلاتس وتغيير جريد 1</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7416,56 +6312,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>13\10\2025</t>
@@ -7486,11 +6342,7 @@
           <t>تم تغيير الجرائد الخلفيه (1_5_8)</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7498,56 +6350,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>30\11\2025</t>
@@ -7568,11 +6380,7 @@
           <t>تم سن الفلاتس</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7580,56 +6388,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -7650,11 +6418,7 @@
           <t>تم تغير سير  دوبل700(محمد نعيم)</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7662,56 +6426,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -7732,11 +6456,7 @@
           <t>تم تغير سوفت كرد لbc</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7744,56 +6464,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -7814,11 +6494,7 @@
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7826,56 +6502,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -7896,11 +6532,7 @@
           <t>تم تغيير  سير 1200 الدوفر المسنن للتجربه</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7908,56 +6540,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>8\3\2026</t>
@@ -7978,11 +6570,7 @@
           <t>تم تبديل اغطيه دوفر بكرد12</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7990,56 +6578,16 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>16/3/2026</t>
@@ -8060,11 +6608,7 @@
           <t>تم تغير سير1200</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -16832,7 +15376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16928,18 +15472,66 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -16957,26 +15549,66 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>21\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16994,18 +15626,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17023,7 +15703,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17039,22 +15723,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>19\1\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17077,25 +15785,61 @@
           <t>573</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>8\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17118,16 +15862,36 @@
           <t>729</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17138,9 +15902,21 @@
           <t>7\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17168,12 +15944,36 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -17189,7 +15989,11 @@
           <t>تم سن الفلاتس لاول مره بعد التغير</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17212,7 +16016,11 @@
           <t>869</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -17223,18 +16031,46 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>30\9\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17257,21 +16093,41 @@
           <t>1059</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -17309,18 +16165,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17338,18 +16242,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17367,18 +16319,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17386,16 +16386,56 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>7/1/2026</t>
@@ -17423,16 +16463,56 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -17460,16 +16540,56 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -17488,6 +16608,63 @@
       <c r="O16" t="inlineStr">
         <is>
           <t>تم تشحيم السلندر  15جرام كل جانب   والدوفر 7 جرام كل جانب</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1226</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>16/3/2026</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>م.عبدالله،محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>تم سن فلاتس وتغير جريده خلفيه240,320</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة صف جديد في Card9 by admin at 2026-03-17 06:15:31
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -9106,7 +9106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9207,19 +9207,71 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9252,20 +9304,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>21\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9283,19 +9371,71 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9313,7 +9453,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9329,23 +9473,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>28\1\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9368,26 +9540,66 @@
           <t>578</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>13\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9410,16 +9622,36 @@
           <t>749</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9430,10 +9662,26 @@
           <t>19\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9456,7 +9704,11 @@
           <t>880</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -9467,19 +9719,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>5\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9507,25 +9791,61 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>26/11/2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>م محمد عبدالله ،ف.محمود ايهاب</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9543,19 +9863,71 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9573,19 +9945,71 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9603,19 +10027,71 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9623,16 +10099,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>20/9/2025</t>
@@ -9653,7 +10169,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9661,16 +10181,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>21\7\2025</t>
@@ -9691,7 +10251,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9699,22 +10263,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه + عمل صيانه</t>
@@ -9725,7 +10333,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9733,22 +10345,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>25\8\2024</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>تم عمل معايره للمكنه setting</t>
@@ -9759,7 +10415,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9767,22 +10427,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\10\2024</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -9793,7 +10497,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9801,22 +10509,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>14\10\2024</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>تم تغيير السستم من ax الي ay</t>
@@ -9827,7 +10579,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9835,22 +10591,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>31\12\2025</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -9861,7 +10661,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9869,22 +10673,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>9\1\2025</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم عمل معايره وصيانه نصف سنويه</t>
@@ -9895,7 +10743,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9903,16 +10755,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>23/11/2025</t>
@@ -9933,7 +10825,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9941,22 +10837,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>18\1\2025</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>تم سن الفلاتس والسليندر ومعايره المكنه وتغيير الجرائد الخلفيه (1_5_8)</t>
@@ -9967,7 +10907,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9975,22 +10919,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>13\4\2025</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه(1_2_4_5_7_8)</t>
@@ -10001,7 +10989,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10009,22 +11001,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>24\4\2025</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>تم تغيير شداد السليندر والليكران والشداد العلوي</t>
@@ -10035,7 +11071,11 @@
           <t>م\محمد عبدالله</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10043,22 +11083,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>10\7\2025</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>تم تغيير زيت الجيربوكس</t>
@@ -10069,7 +11153,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10077,22 +11165,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>19\7\2025</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>تم تغيير الفلاتس وجريده 1</t>
@@ -10103,7 +11235,11 @@
           <t>الخبير محمود رشدي</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10111,22 +11247,66 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>19\7\2025</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>تم تغير الجرائد الخلفيه (1_5_8)</t>
@@ -10137,7 +11317,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10145,16 +11329,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>26\11\2025</t>
@@ -10175,7 +11399,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10183,16 +11411,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>9/12/2025</t>
@@ -10240,30 +11508,66 @@
           <t>1035</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>9/12/2025</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr">
         <is>
           <t xml:space="preserve">م محمد عبدالله </t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10271,16 +11575,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -10301,7 +11645,11 @@
           <t>م. احمد علي توكيل</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10309,16 +11657,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>23/1/2026</t>
@@ -10339,7 +11727,11 @@
           <t>فني ورديه</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10347,16 +11739,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>26/1/2026</t>
@@ -10377,7 +11809,11 @@
           <t>سلامه (محمد عبدالرحمن)</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10385,16 +11821,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -10415,7 +11891,11 @@
           <t>يوسف وابراهيم</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10423,16 +11903,56 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>4/3/2026</t>
@@ -10453,7 +11973,69 @@
           <t>محمود ايهاب</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1125</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>24/2/2026</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تغير جرائد خلفيه بالكامل </t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>م.عبدالله،ايهاب،حسام</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15472,66 +17054,18 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15549,66 +17083,26 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>21\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15626,66 +17120,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15703,11 +17149,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -15723,46 +17165,22 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>19\1\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15785,61 +17203,25 @@
           <t>573</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>8\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15862,36 +17244,16 @@
           <t>729</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -15902,21 +17264,9 @@
           <t>7\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15944,36 +17294,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>6/11/2025</t>
@@ -15989,11 +17315,7 @@
           <t>تم سن الفلاتس لاول مره بعد التغير</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16016,11 +17338,7 @@
           <t>869</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>✔</t>
@@ -16031,46 +17349,18 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>30\9\2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16093,41 +17383,21 @@
           <t>1059</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -16165,66 +17435,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16242,66 +17464,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16319,66 +17493,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16386,56 +17512,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>7/1/2026</t>
@@ -16463,56 +17549,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>19/1/2026</t>
@@ -16540,56 +17586,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>18/2/2026</t>

</xml_diff>

<commit_message>
إضافة صف جديد في Card9 by admin at 2026-03-17 09:40:57
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -9106,7 +9106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12000,7 +12000,11 @@
           <t>1125</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>✅</t>
@@ -12011,10 +12015,26 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>24/2/2026</t>
@@ -12035,7 +12055,65 @@
           <t>م.عبدالله،ايهاب،حسام</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1151</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1160</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>17/3/2026</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>تم سن فلاتس</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>م.عبدالله،ايهاب</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل حدث في Card20 - الصف 39 by admin at 2026-03-25 06:15:31
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -26291,16 +26291,56 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>24/2/2026</t>

</xml_diff>

<commit_message>
إضافة صف جديد في Card20 by admin at 2026-03-25 06:16:47
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -23002,7 +23002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26361,7 +26361,65 @@
           <t>محمود ايهاب</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1150</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1144</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>24/2/2026</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>تم تغير جريده خلفيه240,320</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>محمود ايهاب ،م.عبدالله</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card20 by admin at 2026-03-25 06:19:10
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -23632,27 +23632,27 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>17/12/2025</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>سيرفيس</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t xml:space="preserve">تم تغير فلاتس متحرك </t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>تيم كرد</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -26388,17 +26388,41 @@
           <t>1144</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>24/2/2026</t>
@@ -26419,7 +26443,11 @@
           <t>محمود ايهاب ،م.عبدالله</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card19 by admin at 2026-03-29 13:25:42
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -24696,7 +24696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24792,18 +24792,66 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24821,26 +24869,66 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>5\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24858,18 +24946,66 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24887,18 +25023,66 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24921,9 +25105,21 @@
           <t>595</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -24934,16 +25130,36 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>30\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -24966,25 +25182,61 @@
           <t>797</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>23\8\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25007,16 +25259,36 @@
           <t>994</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>✅</t>
@@ -25027,8 +25299,16 @@
           <t>17/12/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،تيم الكرد</t>
@@ -25056,17 +25336,41 @@
           <t>1076</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>1/2/2026</t>
@@ -25104,18 +25408,66 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25133,18 +25485,66 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -25162,18 +25562,66 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -25181,22 +25629,66 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>10\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -25214,22 +25706,66 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>10\12\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -25247,22 +25783,66 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>5\12\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>تم سن الفلاتس</t>
@@ -25280,16 +25860,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>30\4\2025</t>
@@ -25317,16 +25937,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\8\2025</t>
@@ -25354,16 +26014,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>23\8\2025</t>
@@ -25391,16 +26091,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>26\10\2025</t>
@@ -25428,16 +26168,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -25465,16 +26245,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>17/7/2025</t>
@@ -25502,16 +26322,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>17/12/2025</t>
@@ -25539,16 +26399,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>23/1/2026</t>
@@ -25576,16 +26476,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>14/2/2026</t>
@@ -25613,16 +26553,56 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>17/2/2026</t>
@@ -25641,6 +26621,43 @@
       <c r="O25" t="inlineStr">
         <is>
           <t>رضا واسلام</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>28/3/2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>قطع سير ناقل حركه من دوفر لمجموعه شاشه</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>تم تغير سير</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>سعيد</t>
         </is>
       </c>
     </row>
@@ -28186,76 +29203,20 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -28273,11 +29234,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -28288,61 +29245,21 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>25\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -28360,76 +29277,28 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>23\1\2025</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28452,71 +29321,27 @@
           <t>497</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>23\4\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -28539,71 +29364,27 @@
           <t>696</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>13\8\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -28626,11 +29407,7 @@
           <t>808</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t xml:space="preserve"> ✔</t>
@@ -28641,56 +29418,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>21\10\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -28713,21 +29454,13 @@
           <t>945</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -28738,11 +29471,7 @@
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -28768,16 +29497,8 @@
           <t>م.عبدالله،حسام،ايهاب،سعيد</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -28800,41 +29521,13 @@
           <t>1033</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>26/2/2026</t>
@@ -28855,11 +29548,7 @@
           <t xml:space="preserve">م.سامر.م.محمد عبدالله.محمود إيهاب.حسام .سعيد .محمد ابراهيم </t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -28882,76 +29571,20 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -28969,76 +29602,20 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -29056,76 +29633,20 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -29133,66 +29654,22 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -29203,16 +29680,8 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -29220,66 +29689,22 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>12\12\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -29290,16 +29715,8 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -29307,66 +29724,22 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>25\12\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>تم سن الفلاتس ومعيارها</t>
@@ -29377,16 +29750,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -29394,66 +29759,22 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>10\1\2025</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>تم سن الدوفر</t>
@@ -29464,16 +29785,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -29481,66 +29794,22 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>10\1\2025</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -29551,16 +29820,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -29568,56 +29829,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>23\4\2025</t>
@@ -29638,16 +29859,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -29655,56 +29868,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>13\8\2025</t>
@@ -29725,16 +29898,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -29742,56 +29907,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>21\10\2025</t>
@@ -29812,16 +29937,8 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -29829,56 +29946,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>11/5/2025</t>
@@ -29899,16 +29976,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -29916,56 +29985,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>27/8/2025</t>
@@ -29986,16 +30015,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -30003,56 +30024,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>19/10/2025</t>
@@ -30073,16 +30054,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -30090,56 +30063,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>11/11/2025</t>
@@ -30160,16 +30093,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -30177,56 +30102,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>17/11/2025</t>
@@ -30247,16 +30132,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -30264,56 +30141,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>18/5/2025</t>
@@ -30334,16 +30171,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -30351,56 +30180,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>28/9/2025</t>
@@ -30421,16 +30210,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -30438,56 +30219,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>6/12/2025</t>
@@ -30508,16 +30249,8 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -30525,56 +30258,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>18/12/2025</t>
@@ -30600,11 +30293,7 @@
           <t>IMG-20251218-WA0032_cac4bf63.jpg</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -30612,56 +30301,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>23/12/2025</t>
@@ -30682,16 +30331,8 @@
           <t>عمر</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -30699,56 +30340,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>27/12/2025</t>
@@ -30774,11 +30375,7 @@
           <t>IMG20251227152629_862d6472.jpg, IMG20251227150839_7e109cd6.jpg, IMG20251227150834_e1143419.jpg</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -30786,56 +30383,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>28/1/2026</t>
@@ -30856,16 +30413,8 @@
           <t>ايهاب/مصطفى/م-محمد</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -30873,56 +30422,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>6/2/2026</t>
@@ -30943,16 +30452,8 @@
           <t>م.محمد عبدالله ،محمود ايهاب حسام ،مصطفي</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -30960,56 +30461,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -31030,16 +30491,8 @@
           <t>مصطفى</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -31047,56 +30500,16 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>2/3/2026</t>
@@ -31117,16 +30530,8 @@
           <t>م.رشدي،خبير نور الدين</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card11 by admin at 2026-03-31 09:10:05
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6855,19 +6855,71 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6885,7 +6937,11 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -6896,20 +6952,56 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6927,19 +7019,71 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6957,7 +7101,11 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -6973,19 +7121,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>8\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7008,26 +7188,66 @@
           <t>595</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>17\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7050,20 +7270,36 @@
           <t>764</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7074,10 +7310,26 @@
           <t>21\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7100,7 +7352,11 @@
           <t>899</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7111,19 +7367,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>9\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7151,25 +7439,61 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>29/11/2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.محمود ايهاب</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7192,13 +7516,41 @@
           <t>1039</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>22/11/2025</t>
@@ -7219,7 +7571,11 @@
           <t>م.اشرف كهرباء ،ف. سعيد السيد</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7237,19 +7593,67 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1258</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>31/3/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سيرفيس </t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه 240,240,320</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7267,19 +7671,71 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7297,19 +7753,71 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7317,16 +7825,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -7347,7 +7895,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7355,16 +7907,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -7385,7 +7977,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7393,16 +7989,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>16\7\2024</t>
@@ -7423,7 +8059,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7431,22 +8071,66 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -7457,7 +8141,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7465,22 +8153,66 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>19\10\2024</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -7491,7 +8223,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7499,22 +8235,66 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>8\3\2025</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -7525,7 +8305,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7533,22 +8317,66 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>17\4\2025</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه (1_2_4_5_7_8)</t>
@@ -7559,7 +8387,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7567,16 +8399,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -7597,7 +8469,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7605,16 +8481,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>10\11\2025</t>
@@ -7635,7 +8551,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7643,16 +8563,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>10\11\2025</t>
@@ -7673,7 +8633,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7681,16 +8645,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>21\7\2025</t>
@@ -7711,7 +8715,11 @@
           <t>الخبير محمود رشدي</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7719,16 +8727,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>9\10\2025</t>
@@ -7749,7 +8797,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7757,16 +8809,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>29\11\2025</t>
@@ -7787,7 +8879,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7795,16 +8891,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>3/1/2026</t>
@@ -7825,7 +8961,11 @@
           <t>حسام</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7833,16 +8973,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -7863,7 +9043,11 @@
           <t>م. احمد علي توكيل</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7886,21 +9070,41 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>9/2/2026</t>
@@ -7921,7 +9125,11 @@
           <t>م.محمد عبدالله ،محمود ايهاب ،مصطفي</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7929,16 +9137,56 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -7959,7 +9207,11 @@
           <t>يوسف وابراهيم</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24792,66 +26044,18 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24869,66 +26073,26 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>5\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24946,66 +26110,18 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -25023,66 +26139,18 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -25105,21 +26173,9 @@
           <t>595</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -25130,36 +26186,16 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>30\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -25182,61 +26218,25 @@
           <t>797</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>23\8\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25259,36 +26259,16 @@
           <t>994</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>✅</t>
@@ -25299,16 +26279,8 @@
           <t>17/12/2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،تيم الكرد</t>
@@ -25336,41 +26308,17 @@
           <t>1076</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>1/2/2026</t>
@@ -25408,66 +26356,18 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25485,66 +26385,18 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -25562,66 +26414,18 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -25629,66 +26433,22 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>10\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -25706,66 +26466,22 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>10\12\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -25783,66 +26499,22 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>5\12\2024</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>تم سن الفلاتس</t>
@@ -25860,56 +26532,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>30\4\2025</t>
@@ -25937,56 +26569,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\8\2025</t>
@@ -26014,56 +26606,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>23\8\2025</t>
@@ -26091,56 +26643,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>26\10\2025</t>
@@ -26168,56 +26680,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>5/3/2025</t>
@@ -26245,56 +26717,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>17/7/2025</t>
@@ -26322,56 +26754,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>17/12/2025</t>
@@ -26399,56 +26791,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>23/1/2026</t>
@@ -26476,56 +26828,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>14/2/2026</t>
@@ -26553,56 +26865,16 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>17/2/2026</t>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card17 by admin at 2026-03-31 09:12:50
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6855,71 +6855,19 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6937,11 +6885,7 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
@@ -6952,56 +6896,20 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>16\7\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7019,71 +6927,19 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7101,11 +6957,7 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7121,51 +6973,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>8\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7188,66 +7008,26 @@
           <t>595</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>17\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7270,36 +7050,20 @@
           <t>764</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7310,26 +7074,10 @@
           <t>21\7\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7352,11 +7100,7 @@
           <t>899</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -7367,51 +7111,19 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>9\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7439,61 +7151,25 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>29/11/2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>م.محمد عبدالله ،ف.محمود ايهاب</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7516,41 +7192,13 @@
           <t>1039</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>22/11/2025</t>
@@ -7571,11 +7219,7 @@
           <t>م.اشرف كهرباء ،ف. سعيد السيد</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7609,26 +7253,10 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>31/3/2026</t>
@@ -7649,11 +7277,7 @@
           <t>محمود ايهاب</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7671,71 +7295,19 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7753,71 +7325,19 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7825,56 +7345,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>24/3/2025</t>
@@ -7895,11 +7375,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7907,56 +7383,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -7977,11 +7413,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7989,56 +7421,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>16\7\2024</t>
@@ -8059,11 +7451,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8071,66 +7459,22 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\8\2024</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -8141,11 +7485,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8153,66 +7493,22 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>19\10\2024</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>تم عمل صيانه نصف سنويه</t>
@@ -8223,11 +7519,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8235,66 +7527,22 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>8\3\2025</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>تم سن الفلاتس وتغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -8305,11 +7553,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8317,66 +7561,22 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>17\4\2025</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الاماميه (1_2_4_5_7_8)</t>
@@ -8387,11 +7587,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8399,56 +7595,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>8/11/2025</t>
@@ -8469,11 +7625,7 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8481,56 +7633,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>10\11\2025</t>
@@ -8551,11 +7663,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8563,56 +7671,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>10\11\2025</t>
@@ -8633,11 +7701,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8645,56 +7709,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>21\7\2025</t>
@@ -8715,11 +7739,7 @@
           <t>الخبير محمود رشدي</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8727,56 +7747,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>9\10\2025</t>
@@ -8797,11 +7777,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8809,56 +7785,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>29\11\2025</t>
@@ -8879,11 +7815,7 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8891,56 +7823,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>3/1/2026</t>
@@ -8961,11 +7853,7 @@
           <t>حسام</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8973,56 +7861,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>20/1/2026</t>
@@ -9043,11 +7891,7 @@
           <t>م. احمد علي توكيل</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9070,41 +7914,21 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>9/2/2026</t>
@@ -9125,11 +7949,7 @@
           <t>م.محمد عبدالله ،محمود ايهاب ،مصطفي</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9137,56 +7957,16 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>18/2/2026</t>
@@ -9207,11 +7987,7 @@
           <t>يوسف وابراهيم</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28444,19 +27220,71 @@
           <t>150</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -28474,27 +27302,71 @@
           <t>300</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>9\12\2024</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -28512,19 +27384,71 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28542,8 +27466,16 @@
           <t>550</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>✔</t>
@@ -28554,19 +27486,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>10\3\2025</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -28589,26 +27553,66 @@
           <t>593</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>27\4\2025</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -28631,26 +27635,66 @@
           <t>783</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>14\8\2025</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -28673,7 +27717,11 @@
           <t>894</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>✔</t>
@@ -28684,19 +27732,51 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>22\10\2025</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -28714,19 +27794,71 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -28744,19 +27876,71 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1169</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>30/3/2026</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سيرفبس </t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه بالكامل 240,240,320</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">م.عبدالله،محمود ايهاب </t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -28774,19 +27958,71 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -28804,19 +28040,71 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -28824,22 +28112,66 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>13\8\2024</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>تم تشحيم المكنه بالكامل +عمل صيانه</t>
@@ -28850,7 +28182,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -28858,22 +28194,66 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>9\12\2024</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>تم سن الفلاتس + صينه نصف سنويه</t>
@@ -28884,7 +28264,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -28892,22 +28276,66 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>10\3\2025</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الخلفيه (1_5_8) ومعايره</t>
@@ -28918,7 +28346,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -28926,16 +28358,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>27\4\2025</t>
@@ -28956,7 +28428,11 @@
           <t>الخبير</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -28964,22 +28440,66 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>14\8\2025</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>تم تغيير زيت الجيربوكس</t>
@@ -28990,7 +28510,11 @@
           <t>تيم العمل</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -28998,22 +28522,66 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>22\10\2025</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>تم تغيير الجرائد الخلفيه (1_5_8) ومعايرتها</t>
@@ -29024,7 +28592,11 @@
           <t>م\محمد عبدالله</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -29032,16 +28604,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>9/9/2025</t>
@@ -29062,7 +28674,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -29070,16 +28686,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>16/9/2025</t>
@@ -29100,7 +28756,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -29108,16 +28768,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>4/5/2025</t>
@@ -29138,7 +28838,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -29146,16 +28850,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>18/5/2025</t>
@@ -29176,7 +28920,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -29184,16 +28932,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>29/11/2025</t>
@@ -29214,7 +29002,11 @@
           <t>فني</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -29237,20 +29029,36 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t xml:space="preserve">Done </t>
@@ -29288,16 +29096,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>21/2/2026</t>
@@ -29318,7 +29166,11 @@
           <t>مصطفى</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -29326,16 +29178,56 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>25/2/2026</t>
@@ -29356,7 +29248,11 @@
           <t>سعيد</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card21 by admin at 2026-04-04 06:36:45
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -21676,7 +21676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23091,6 +23091,44 @@
       </c>
       <c r="P37" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>31/3/2026</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>قطع سير700</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>تم تغير سيى700(مشلان)</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>حسام</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card11 by admin at 2026-04-04 06:37:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6770,7 +6770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8004,6 +8004,44 @@
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>3/4/2026</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>قطع سيردوفر1200</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>تم تغير سير دوفر1200</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>حسام</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card11 by admin at 2026-04-04 06:39:04
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -6770,7 +6770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8042,6 +8042,44 @@
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>4/4/2026</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>قطع سيردوفر1520</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>تم تغير سير دوفر1520</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>حسام</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card10 by admin at 2026-04-04 16:51:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -8092,7 +8092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9307,6 +9307,43 @@
       <c r="O31" t="inlineStr">
         <is>
           <t>رضا</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>4/4/2026</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>قطع سير كويلر1465</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>تم تغير سير كويلر1465</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>سلامه</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card4 by admin at 2026-04-06 11:37:33
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -12657,18 +12657,46 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1192.5</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>5/4/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه بالكامل 240,240,320</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسام ،م.محمد عبدالله </t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card5 by admin at 2026-04-06 11:39:00
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -15406,18 +15406,46 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1178</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>6/4/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه بالكامل 240,240,320</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>م.محمد عبدالله ،مصطفي،محمود ايهاب،حسام</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card6 by admin at 2026-04-07 16:01:55
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -14628,18 +14628,46 @@
           <t>450</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>7/4/2026</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه بالكامل240,240,320</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>محمد عبدالله ،محمود ايهاب</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
إضافة صف جديد في Card7 by admin at 2026-04-08 12:22:41
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -11611,7 +11611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12158,6 +12158,63 @@
       <c r="O15" t="inlineStr">
         <is>
           <t>يوسف وابراهيم</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>8/4/2023</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>سيرفس</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد الخلفيه 240,240,320</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>م.عبدالله،حسام ،محمود ايهاب</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card17 by admin at 2026-04-09 13:05:01
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -27455,7 +27455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28497,6 +28497,44 @@
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>9/4/2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>قطع سيى1350</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>تم تغير سير1350</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>سعيد</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card17 by admin at 2026-04-09 13:05:44
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -27455,7 +27455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28535,6 +28535,44 @@
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>9/4/2026</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>كسر شفاط جانبي شمال علوي</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>تم لحم الشفاط</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card17 by admin at 2026-04-09 16:10:10
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -28521,12 +28521,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>قطع سيى1350</t>
+          <t>قطع سيىر1200*18*2.5</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>تم تغير سير1350</t>
+          <t>تم تغير سير1200*18*2.5</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card8 by admin at 2026-04-11 12:13:31
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -11307,18 +11307,50 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1228</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>11/4/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>تم سن الفلاتس وتغير جرائد خلفيه بالكامل 240,240,320</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مصطفي،حسام،م.محمد عبدالله </t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11820,21 +11852,9 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card24 by admin at 2026-04-13 08:22:48
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2039,6 +2039,42 @@
           <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20251215142657_49b68bf2.jpg</t>
         </is>
       </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>13/4/2026</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>صوة عالي في مجموعة عصرات الدلڤري</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>6006-2RS1/C3 تم تغيير بليه
+تم تركيب البليه في المجموعة الداخلية</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة حدث جديد في Card24 by admin at 2026-04-13 08:25:34
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2083,6 +2083,45 @@
           <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260413094236_b8eefacf.jpg,https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260413094242_70b7006f.jpg</t>
         </is>
       </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>13/4/2026</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>تلف سير700</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>تم تغير سير700(مشلان)</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>محمود ايهاب</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card13 by admin at 2026-04-15 12:56:42
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -4793,18 +4793,42 @@
           <t>1300</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1190</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>15/4/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه العلوية 240.320</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سيرفس </t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>محمد عبدالله ،محمود ايهاب</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -13518,7 +13542,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>تم اللحام بلحام حديد</t>
+          <t>تم اللحام باستخدام لحام حديد</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -13528,7 +13552,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113558_cbb49cf1.jpg,https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113640_ffc3947d.jpg</t>
+          <t>https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113640_2dc9d667.jpg,https://raw.githubusercontent.com/mahmedabdallh123/BELYARN/main/event_images/IMG20260414113558_f6dff8da.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة عمود جديد 'Cylinder (o)' إلى Card10 by admin at 2026-04-18 21:21:32
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -8313,7 +8313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8390,6 +8390,11 @@
       <c r="O1" t="inlineStr">
         <is>
           <t>Serviced by</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Cylinder (o)</t>
         </is>
       </c>
     </row>
@@ -8421,6 +8426,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8462,6 +8468,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8491,6 +8498,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8540,6 +8548,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8581,6 +8590,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8630,6 +8640,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8675,6 +8686,7 @@
           <t>م.محمد عبدالله ،ف.مصطفي</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8720,6 +8732,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8777,6 +8790,7 @@
           <t>م.محمد,عمر,محمود ايهاب</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8806,6 +8820,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8835,6 +8850,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8864,6 +8880,7 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8901,6 +8918,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8938,6 +8956,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8975,6 +8994,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9012,6 +9032,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9049,6 +9070,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9086,6 +9108,7 @@
           <t>فني</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9119,6 +9142,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9152,6 +9176,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9185,6 +9210,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9218,6 +9244,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9255,6 +9282,7 @@
           <t>تيم العمل</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9288,6 +9316,7 @@
           <t>الخبير محمود رشدي</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9325,6 +9354,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9362,6 +9392,7 @@
           <t>الخبير</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9399,6 +9430,7 @@
           <t>م. احمد علي توكيل</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9456,6 +9488,7 @@
           <t xml:space="preserve">م.محمد عبدالله ،محمود ايهاب </t>
         </is>
       </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9493,6 +9526,7 @@
           <t>يوسف وابراهيم</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9530,6 +9564,7 @@
           <t>رضا</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9567,6 +9602,7 @@
           <t>سلامه</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
إضافة صف جديد في Card21 by admin at 2026-04-20 07:31:31
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -22381,7 +22381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23930,6 +23930,65 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1150</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1116</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>12/3/2026</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>سيرفيس</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>تم تغير جرائد خلفيه بالكامل 320,240,240</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>م.عبدالله،ايهاب</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>